<commit_message>
Documents engine: validate files before writes, dedup document per object+type
- File read/validated before any Loodsman writes (folder/document/link
  no longer created for a row whose file is missing or unreadable).
- One "Бумажный документ" per (object name, document type) instead of
  per row — multiple files of the same type attach to the same
  document via repeated File/add calls.
- New documentTypeColumn (the previously-unused second column from the
  original spec) written to the "Тип документа" attribute; key
  attribute becomes "<object name> - <document type>" for uniqueness.
  Blank type falls back to "Без типа".
- Updated settings.json and test-data/ to match (per-object scan
  subfolders, second document type per object, blank-type row).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-data/documents.xlsx
+++ b/test-data/documents.xlsx
@@ -422,12 +422,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -438,10 +439,15 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Тип документа</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Расположение файла</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Имя документа</t>
         </is>
@@ -455,10 +461,15 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>/Users/khan/Projects/lis-client-ktor/test-data/scans</t>
+          <t>Чертёж</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>/Users/khan/Projects/lis-client-ktor/test-data/scans/Деталь-001</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>scan1.txt</t>
         </is>
@@ -472,10 +483,15 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>/Users/khan/Projects/lis-client-ktor/test-data/scans</t>
+          <t>Чертёж</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>/Users/khan/Projects/lis-client-ktor/test-data/scans/Деталь-001</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>scan2.txt</t>
         </is>
@@ -484,32 +500,60 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Деталь-002</t>
+          <t>Деталь-001</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>/Users/khan/Projects/lis-client-ktor/test-data/scans</t>
+          <t>Паспорт</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>scan3.txt</t>
+          <t>/Users/khan/Projects/lis-client-ktor/test-data/scans/Деталь-001</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>scan_passport.txt</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>Деталь-002</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>/Users/khan/Projects/lis-client-ktor/test-data/scans/Деталь-002</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>scan3.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>Деталь-003</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>/Users/khan/Projects/lis-client-ktor/test-data/scans</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Чертёж</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>/Users/khan/Projects/lis-client-ktor/test-data/scans/Деталь-003</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>scan4_missing.txt</t>
         </is>

</xml_diff>